<commit_message>
fix final exel file
</commit_message>
<xml_diff>
--- a/IT23633018_Assignment 1 - Test cases.xlsx
+++ b/IT23633018_Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\test_automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\IT23633018-B,A,S,B,SMARATHUNGA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5456118-B6E1-4B39-8EC8-62CC3A5F3FE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1928A22-6E30-4A66-BA96-514B1C7A0DEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="288">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -582,12 +582,318 @@
   </si>
   <si>
     <t>wඉෆි පස්සwඔර්ඩ් එක මොකක්ඩ?</t>
+  </si>
+  <si>
+    <t>Accuracy justification/ Description of issue type</t>
+  </si>
+  <si>
+    <t>What is covered by the test</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>The greeting meaning is preserved and the output matches the expected Sinhala sentence.</t>
+  </si>
+  <si>
+    <t>Question meaning is preserved and the output matches the expected Sinhala sentence.</t>
+  </si>
+  <si>
+    <t>Request sentence is translated correctly and matches the expected output.</t>
+  </si>
+  <si>
+    <t>Command/request meaning is translated correctly and matches the expected output.</t>
+  </si>
+  <si>
+    <t>Greeting meaning and exclamation mark are preserved correctly.</t>
+  </si>
+  <si>
+    <t>Friendly greeting sentence is translated correctly.</t>
+  </si>
+  <si>
+    <t>English loan word “phone” is not converted to the expected Sinhala form.</t>
+  </si>
+  <si>
+    <t>Question meaning and question mark are preserved correctly.</t>
+  </si>
+  <si>
+    <t>Positive confirmation meaning is translated correctly.</t>
+  </si>
+  <si>
+    <t>Negative response meaning is translated correctly.</t>
+  </si>
+  <si>
+    <t>Repeated informal phrase and sentence meaning are preserved.</t>
+  </si>
+  <si>
+    <t>Repeated question phrase and question mark are preserved.</t>
+  </si>
+  <si>
+    <t>Emotion word and punctuation are preserved correctly.</t>
+  </si>
+  <si>
+    <t>Actual output is not generated/displayed by the UI.</t>
+  </si>
+  <si>
+    <t>Informal shortened Sinhala text is converted incorrectly.</t>
+  </si>
+  <si>
+    <t>Misspelled informal input is converted into incorrect Sinhala text.</t>
+  </si>
+  <si>
+    <t>Mixed Sinhala-English word “class” is not handled as expected.</t>
+  </si>
+  <si>
+    <t>English word “lunch” is incorrectly converted into Sinhala letters.</t>
+  </si>
+  <si>
+    <t>Long mixed Sinhala-English sentence is poorly converted.</t>
+  </si>
+  <si>
+    <t>Medium mixed sentence contains incorrect Sinhala characters and English words.</t>
+  </si>
+  <si>
+    <t>Technical words “WiFi password” are not handled correctly.</t>
+  </si>
+  <si>
+    <t>Technical words are preserved correctly and output matches expected.</t>
+  </si>
+  <si>
+    <t>Platform name and mixed Sinhala-English sentence are handled correctly.</t>
+  </si>
+  <si>
+    <t>App name and call phrase are preserved correctly.</t>
+  </si>
+  <si>
+    <t>Output is close, but Sinhala wording differs from expected.</t>
+  </si>
+  <si>
+    <t>Technical abbreviation and number are preserved correctly.</t>
+  </si>
+  <si>
+    <t>Exam-related sentence meaning is preserved correctly.</t>
+  </si>
+  <si>
+    <t>Meaning is similar, but Sinhala wording differs from expected.</t>
+  </si>
+  <si>
+    <t>Place name is preserved correctly and output matches expected.</t>
+  </si>
+  <si>
+    <t>Location and transport question is translated correctly.</t>
+  </si>
+  <si>
+    <t>Meaning is similar, but expected wording uses a different Sinhala form.</t>
+  </si>
+  <si>
+    <t>Name and relationship meaning are translated correctly.</t>
+  </si>
+  <si>
+    <t>Number with Sinhala suffix is handled correctly.</t>
+  </si>
+  <si>
+    <t>Ordinal number and English words are not converted in the expected format.</t>
+  </si>
+  <si>
+    <t>Currency amount is preserved, but Sinhala wording is incorrect.</t>
+  </si>
+  <si>
+    <t>Foreign currency value is preserved, but Sinhala wording is incorrect.</t>
+  </si>
+  <si>
+    <t>Time value is preserved, but mixed Sinhala-English wording is incorrect.</t>
+  </si>
+  <si>
+    <t>Time value is preserved, but Sinhala conversion is incorrect.</t>
+  </si>
+  <si>
+    <t>Date value is preserved, but English word conversion is incorrect.</t>
+  </si>
+  <si>
+    <t>Month and number are preserved, but Sinhala wording is incorrect.</t>
+  </si>
+  <si>
+    <t>Distance unit is preserved, but Sinhala word conversion is incorrect.</t>
+  </si>
+  <si>
+    <t>Weight unit is preserved, but Sinhala word conversion is incorrect.</t>
+  </si>
+  <si>
+    <t>Informal Sinhala slang meaning is preserved correctly.</t>
+  </si>
+  <si>
+    <t>English word “dial” is not converted to the expected Sinhala form.</t>
+  </si>
+  <si>
+    <t>URL and mixed English words are preserved correctly.</t>
+  </si>
+  <si>
+    <t>Email address and mixed English words are preserved correctly.</t>
+  </si>
+  <si>
+    <t>Meaning is preserved; only trailing space difference exists.</t>
+  </si>
+  <si>
+    <t>Emotion sentence is incomplete and Sinhala wording is inaccurate.</t>
+  </si>
+  <si>
+    <t>Long sentence with time, app names, and link wording is inaccurately converted.</t>
+  </si>
+  <si>
+    <t>· Greeting / request / response; · S (≤30 characters); · Question sentence</t>
+  </si>
+  <si>
+    <t>· Emotional question; · S (≤30 characters); · Interrogative sentence</t>
+  </si>
+  <si>
+    <t>· Simple request sentence; · S (≤30 characters); · Object/request translation</t>
+  </si>
+  <si>
+    <t>· Command sentence; · S (≤30 characters); · Direction/action meaning</t>
+  </si>
+  <si>
+    <t>· Greeting with punctuation; · S (≤30 characters); · Exclamation mark handling</t>
+  </si>
+  <si>
+    <t>· Friendly greeting sentence; · S (≤30 characters); · Informal Sinhala greeting</t>
+  </si>
+  <si>
+    <t>· English loan word handling; · S (≤30 characters); · Mixed Sinhala-English word</t>
+  </si>
+  <si>
+    <t>· Question sentence; · S (≤30 characters); · Question mark handling</t>
+  </si>
+  <si>
+    <t>· Positive response sentence; · S (≤30 characters); · Confirmation meaning</t>
+  </si>
+  <si>
+    <t>· Negative response sentence; · S (≤30 characters); · Rejection/negative meaning</t>
+  </si>
+  <si>
+    <t>· Repeated informal phrase; · S (≤30 characters); · Casual Sinhala expression</t>
+  </si>
+  <si>
+    <t>· Repeated question phrase; · S (≤30 characters); · Interrogative repetition</t>
+  </si>
+  <si>
+    <t>· Emotion and punctuation handling; · S (≤30 characters); · Exclamation sentence</t>
+  </si>
+  <si>
+    <t>· UI output validation; · S (≤30 characters); · Missing/blank actual output</t>
+  </si>
+  <si>
+    <t>· Shortened informal typing; · S (≤30 characters); · Informal input handling</t>
+  </si>
+  <si>
+    <t>· Misspelled informal input; · S (≤30 characters); · Typing error handling</t>
+  </si>
+  <si>
+    <t>· Mixed Sinhala-English word; · S (≤30 characters); · English word preservation</t>
+  </si>
+  <si>
+    <t>· English food word handling; · S (≤30 characters); · Loan word conversion</t>
+  </si>
+  <si>
+    <t>· Mixed Sinhala-English sentence; · M (31–100 characters); · Long sentence handling</t>
+  </si>
+  <si>
+    <t>· Mixed Sinhala-English sentence; · M (31–100 characters); · Future action meaning</t>
+  </si>
+  <si>
+    <t>· Technical word handling; · S (≤30 characters); · WiFi/password term</t>
+  </si>
+  <si>
+    <t>· Technical word handling; · S (≤30 characters); · Email/link term</t>
+  </si>
+  <si>
+    <t>· Platform name handling; · S (≤30 characters); · Zoom class phrase</t>
+  </si>
+  <si>
+    <t>· App name handling; · S (≤30 characters); · WhatsApp call phrase</t>
+  </si>
+  <si>
+    <t>· File format handling; · S (≤30 characters); · PDF/CV wording</t>
+  </si>
+  <si>
+    <t>· ID number handling; · S (≤30 characters); · NIC number phrase</t>
+  </si>
+  <si>
+    <t>· Exam-related sentence; · S (≤30 characters); · Time/place action</t>
+  </si>
+  <si>
+    <t>· Education-related sentence; · S (≤30 characters); · Cancel action meaning</t>
+  </si>
+  <si>
+    <t>· Place name handling; · S (≤30 characters); · Kandy location phrase</t>
+  </si>
+  <si>
+    <t>· Transport question; · S (≤30 characters); · Colombo bus phrase</t>
+  </si>
+  <si>
+    <t>· Personal name sentence; · S (≤30 characters); · Name preservation</t>
+  </si>
+  <si>
+    <t>· Relationship sentence; · S (≤30 characters); · Friend/person meaning</t>
+  </si>
+  <si>
+    <t>· Number handling; · S (≤30 characters); · 2k amount phrase</t>
+  </si>
+  <si>
+    <t>· Ordinal/floor handling; · S (≤30 characters); · English number + floor term</t>
+  </si>
+  <si>
+    <t>· Currency amount handling; · S (≤30 characters); · Rs. 500 phrase</t>
+  </si>
+  <si>
+    <t>· Foreign currency handling; · S (≤30 characters); · USD amount phrase</t>
+  </si>
+  <si>
+    <t>· Time format handling; · S (≤30 characters); · AM time phrase</t>
+  </si>
+  <si>
+    <t>· Time format handling; · S (≤30 characters); · PM time phrase</t>
+  </si>
+  <si>
+    <t>· Date format handling; · S (≤30 characters); · Numeric date phrase</t>
+  </si>
+  <si>
+    <t>· Month and number handling; · S (≤30 characters); · Month name phrase</t>
+  </si>
+  <si>
+    <t>· Distance unit handling; · S (≤30 characters); · KM value phrase</t>
+  </si>
+  <si>
+    <t>· Weight unit handling; · S (≤30 characters); · KG value phrase</t>
+  </si>
+  <si>
+    <t>· Informal Sinhala slang; · S (≤30 characters); · Casual expression</t>
+  </si>
+  <si>
+    <t>· Informal English/Sinhala slang; · S (≤30 characters); · Dial/call wording</t>
+  </si>
+  <si>
+    <t>· URL handling; · S (≤30 characters); · Link/domain preservation</t>
+  </si>
+  <si>
+    <t>· Email address handling; · S (≤30 characters); · Email format preservation</t>
+  </si>
+  <si>
+    <t>· Trailing space handling; · S (≤30 characters); · Extra space validation</t>
+  </si>
+  <si>
+    <t>· Emotion sentence handling; · S (≤30 characters); · Sadness/emotion phrase</t>
+  </si>
+  <si>
+    <t>· Long mixed Sinhala-English sentence; · L (&gt;100 characters); · Complex sentence handling</t>
+  </si>
+  <si>
+    <t>· Long sentence with app/time/link words; · L (&gt;100 characters); · Mixed technical content</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -708,7 +1014,9 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Table Style 1" pivot="0" count="0" xr9:uid="{0BCE0B85-6019-42D8-B673-11BC14888DD4}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -718,6 +1026,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{3CEBF5AB-E727-4E4F-94C2-9DA262CF77A8}" name="Table6" displayName="Table6" ref="A1:H51" totalsRowShown="0">
+  <autoFilter ref="A1:H51" xr:uid="{3CEBF5AB-E727-4E4F-94C2-9DA262CF77A8}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{2B99F3C4-FCE7-4918-8299-C33E7E1C06B3}" name="Column1"/>
+    <tableColumn id="2" xr3:uid="{BE4317C0-E5E3-4D85-A710-E91CCC6A5669}" name="Input length type"/>
+    <tableColumn id="3" xr3:uid="{431DE9BA-9FF0-45F2-8685-A5BAB2ED6D32}" name="Input"/>
+    <tableColumn id="4" xr3:uid="{0175C77C-BAC3-4413-8B15-B431AD1A0A5E}" name="Expected output"/>
+    <tableColumn id="5" xr3:uid="{006FB470-943E-4816-A89E-A3FD798C178D}" name="Actual output"/>
+    <tableColumn id="6" xr3:uid="{2ED46B65-884B-41A5-9B4C-1961B7DBEE79}" name="Status"/>
+    <tableColumn id="7" xr3:uid="{896E3EFA-7658-4CAF-B0A9-593C7C822041}" name="Accuracy justification/ Description of issue type"/>
+    <tableColumn id="8" xr3:uid="{54A40AED-3E7A-4AE0-9EC6-792E86AAC470}" name="What is covered by the test"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -983,7 +1308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -992,11 +1317,12 @@
     <col min="4" max="4" width="71.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="69.5703125" customWidth="1"/>
     <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="80.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>188</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1013,8 +1339,14 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>186</v>
+      </c>
+      <c r="H1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1033,8 +1365,14 @@
       <c r="F2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1053,8 +1391,14 @@
       <c r="F3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>190</v>
+      </c>
+      <c r="H3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1073,8 +1417,14 @@
       <c r="F4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>191</v>
+      </c>
+      <c r="H4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1093,8 +1443,14 @@
       <c r="F5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>192</v>
+      </c>
+      <c r="H5" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1113,8 +1469,14 @@
       <c r="F6" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>193</v>
+      </c>
+      <c r="H6" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1133,8 +1495,14 @@
       <c r="F7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H7" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1153,8 +1521,14 @@
       <c r="F8" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>195</v>
+      </c>
+      <c r="H8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1173,8 +1547,14 @@
       <c r="F9" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>196</v>
+      </c>
+      <c r="H9" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -1193,8 +1573,14 @@
       <c r="F10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>197</v>
+      </c>
+      <c r="H10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>37</v>
       </c>
@@ -1213,8 +1599,14 @@
       <c r="F11" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>198</v>
+      </c>
+      <c r="H11" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -1233,8 +1625,14 @@
       <c r="F12" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>199</v>
+      </c>
+      <c r="H12" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -1253,8 +1651,14 @@
       <c r="F13" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>200</v>
+      </c>
+      <c r="H13" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -1273,8 +1677,14 @@
       <c r="F14" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>201</v>
+      </c>
+      <c r="H14" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>49</v>
       </c>
@@ -1290,8 +1700,14 @@
       <c r="F15" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>202</v>
+      </c>
+      <c r="H15" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>53</v>
       </c>
@@ -1310,8 +1726,14 @@
       <c r="F16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" t="s">
+        <v>203</v>
+      </c>
+      <c r="H16" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>56</v>
       </c>
@@ -1330,8 +1752,14 @@
       <c r="F17" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>204</v>
+      </c>
+      <c r="H17" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>59</v>
       </c>
@@ -1350,8 +1778,14 @@
       <c r="F18" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" t="s">
+        <v>205</v>
+      </c>
+      <c r="H18" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -1370,8 +1804,14 @@
       <c r="F19" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>206</v>
+      </c>
+      <c r="H19" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>65</v>
       </c>
@@ -1390,8 +1830,14 @@
       <c r="F20" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>207</v>
+      </c>
+      <c r="H20" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>69</v>
       </c>
@@ -1410,8 +1856,14 @@
       <c r="F21" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>208</v>
+      </c>
+      <c r="H21" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>72</v>
       </c>
@@ -1430,8 +1882,14 @@
       <c r="F22" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G22" t="s">
+        <v>209</v>
+      </c>
+      <c r="H22" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>75</v>
       </c>
@@ -1450,8 +1908,14 @@
       <c r="F23" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>210</v>
+      </c>
+      <c r="H23" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>78</v>
       </c>
@@ -1470,8 +1934,14 @@
       <c r="F24" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>211</v>
+      </c>
+      <c r="H24" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>81</v>
       </c>
@@ -1490,8 +1960,14 @@
       <c r="F25" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" t="s">
+        <v>212</v>
+      </c>
+      <c r="H25" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>84</v>
       </c>
@@ -1510,8 +1986,14 @@
       <c r="F26" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>213</v>
+      </c>
+      <c r="H26" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>88</v>
       </c>
@@ -1530,8 +2012,14 @@
       <c r="F27" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27" t="s">
+        <v>214</v>
+      </c>
+      <c r="H27" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>91</v>
       </c>
@@ -1550,8 +2038,14 @@
       <c r="F28" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>215</v>
+      </c>
+      <c r="H28" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>94</v>
       </c>
@@ -1570,8 +2064,14 @@
       <c r="F29" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>216</v>
+      </c>
+      <c r="H29" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>98</v>
       </c>
@@ -1590,8 +2090,14 @@
       <c r="F30" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" t="s">
+        <v>217</v>
+      </c>
+      <c r="H30" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>101</v>
       </c>
@@ -1610,8 +2116,14 @@
       <c r="F31" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" t="s">
+        <v>218</v>
+      </c>
+      <c r="H31" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>104</v>
       </c>
@@ -1630,8 +2142,14 @@
       <c r="F32" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>219</v>
+      </c>
+      <c r="H32" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>108</v>
       </c>
@@ -1650,8 +2168,14 @@
       <c r="F33" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" t="s">
+        <v>220</v>
+      </c>
+      <c r="H33" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>111</v>
       </c>
@@ -1670,8 +2194,14 @@
       <c r="F34" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" t="s">
+        <v>221</v>
+      </c>
+      <c r="H34" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>114</v>
       </c>
@@ -1690,8 +2220,14 @@
       <c r="F35" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" t="s">
+        <v>222</v>
+      </c>
+      <c r="H35" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>117</v>
       </c>
@@ -1710,8 +2246,14 @@
       <c r="F36" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36" t="s">
+        <v>223</v>
+      </c>
+      <c r="H36" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>120</v>
       </c>
@@ -1730,8 +2272,14 @@
       <c r="F37" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" t="s">
+        <v>224</v>
+      </c>
+      <c r="H37" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>123</v>
       </c>
@@ -1750,8 +2298,14 @@
       <c r="F38" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>225</v>
+      </c>
+      <c r="H38" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>126</v>
       </c>
@@ -1770,8 +2324,14 @@
       <c r="F39" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" t="s">
+        <v>226</v>
+      </c>
+      <c r="H39" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>129</v>
       </c>
@@ -1790,8 +2350,14 @@
       <c r="F40" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" t="s">
+        <v>227</v>
+      </c>
+      <c r="H40" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>132</v>
       </c>
@@ -1810,8 +2376,14 @@
       <c r="F41" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" t="s">
+        <v>228</v>
+      </c>
+      <c r="H41" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>135</v>
       </c>
@@ -1830,8 +2402,14 @@
       <c r="F42" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" t="s">
+        <v>229</v>
+      </c>
+      <c r="H42" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>138</v>
       </c>
@@ -1850,8 +2428,14 @@
       <c r="F43" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" t="s">
+        <v>230</v>
+      </c>
+      <c r="H43" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>141</v>
       </c>
@@ -1870,8 +2454,14 @@
       <c r="F44" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44" t="s">
+        <v>231</v>
+      </c>
+      <c r="H44" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>144</v>
       </c>
@@ -1890,8 +2480,14 @@
       <c r="F45" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45" t="s">
+        <v>232</v>
+      </c>
+      <c r="H45" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>148</v>
       </c>
@@ -1910,8 +2506,14 @@
       <c r="F46" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46" t="s">
+        <v>233</v>
+      </c>
+      <c r="H46" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>151</v>
       </c>
@@ -1930,8 +2532,14 @@
       <c r="F47" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47" t="s">
+        <v>234</v>
+      </c>
+      <c r="H47" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>154</v>
       </c>
@@ -1950,8 +2558,14 @@
       <c r="F48" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48" t="s">
+        <v>235</v>
+      </c>
+      <c r="H48" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>158</v>
       </c>
@@ -1970,8 +2584,14 @@
       <c r="F49" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G49" t="s">
+        <v>236</v>
+      </c>
+      <c r="H49" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>161</v>
       </c>
@@ -1990,8 +2610,14 @@
       <c r="F50" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G50" t="s">
+        <v>207</v>
+      </c>
+      <c r="H50" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>164</v>
       </c>
@@ -2010,9 +2636,18 @@
       <c r="F51" t="s">
         <v>30</v>
       </c>
+      <c r="G51" t="s">
+        <v>237</v>
+      </c>
+      <c r="H51" t="s">
+        <v>287</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>